<commit_message>
Fill existing abbreviation columns (source -> target) and simplify UI
- No column creation: abbreviations are written into the target column
  the user already has in the file (FillMapping source -> target).
  Missing target, source == target and duplicate targets are errors.
- Multiple columns: tick any number of target columns, pick a source
  for each; '... Abbr' pairs are auto-detected, with Select all / Clear.
- Simple design: 4 clean steps, all fill settings removed (fixed
  defaults), no per-column name/rule inputs, single-sheet download.
- Samples and README updated; 124 tests pass.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/samples/equipment_data.xlsx
+++ b/samples/equipment_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -430,20 +430,35 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Plant Section Abbr</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Equipment Description</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Equipment Description Abbr</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Parameter Abbr</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -458,20 +473,23 @@
           <t>Power House</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Cooling Tower No 2</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="n">
         <v>2</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>old tag: CT-02</t>
         </is>
@@ -486,20 +504,23 @@
           <t>Power House</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
         <is>
           <t>Cooling Tower No.  3</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
         <v>2</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>old tag: CT-03</t>
         </is>
@@ -514,20 +535,23 @@
           <t>Boiler House</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
         <is>
           <t>boiler feed water pump a</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Flow</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>lowercase source data</t>
         </is>
@@ -542,20 +566,23 @@
           <t>Boiler House</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
         <is>
           <t>Boiler Feed Water Pump B</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
         <is>
           <t>Flow</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -566,20 +593,23 @@
           <t>Boiler House</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
         <is>
           <t>Primary Air Fan - 1</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -590,20 +620,23 @@
           <t>Boiler House</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Primary Air Fan - 1</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>exact duplicate of row 5 -&gt; duplicate tag</t>
         </is>
@@ -618,20 +651,23 @@
           <t>Boiler House</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
         <is>
           <t>Primary Air Fan</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -642,20 +678,23 @@
           <t>Boiler House</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Induced Draft Fan</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -666,20 +705,23 @@
           <t>Boiler House</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
         <is>
           <t>Steam Drum Level Transmitter</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -690,20 +732,23 @@
           <t>Boiler House</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
         <is>
           <t xml:space="preserve">   steam   DRUM   pressure   TRANSMITTER  </t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>messy spacing + casing</t>
         </is>
@@ -718,20 +763,23 @@
           <t>Cooling Water System</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
         <is>
           <t>Circulating Water Pump 1</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
         <is>
           <t>Flow</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -742,20 +790,23 @@
           <t>Cooling Water System</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
         <is>
           <t>Circulating Water Pump 2</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
         <is>
           <t>Flow</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -766,20 +817,23 @@
           <t>Water Treatment Plant</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
         <is>
           <t>Raw Water Storage Tank</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -790,20 +844,23 @@
           <t>Water Treatment Plant</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
         <is>
           <t>DM Water Storage Tank</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -814,20 +871,23 @@
           <t>Water Treatment Plant</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
         <is>
           <t>Effluent Treatment Plant Agitator</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>Agitator is not mapped</t>
         </is>
@@ -842,20 +902,23 @@
           <t>Flue Gas System</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
         <is>
           <t>Flue Gas Desulphurisation Unit</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -866,20 +929,23 @@
           <t>Flue Gas System</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
         <is>
           <t>Electrostatic Precipitator</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -890,20 +956,23 @@
           <t>Flue Gas System</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
         <is>
           <t>Scrubber Recirculation Pump</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
         <is>
           <t>Flow</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>Scrubber is not mapped</t>
         </is>
@@ -918,20 +987,23 @@
           <t>Ash Handling</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
         <is>
           <t>Ash Handling Conveyor 3</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
         <is>
           <t>Flow</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -942,20 +1014,23 @@
           <t>Ash Handling</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
         <is>
           <t>Ash Silo Level Indicator</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>Silo is not mapped</t>
         </is>
@@ -970,20 +1045,23 @@
           <t>Turbine Hall</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
         <is>
           <t>Turbine Lube Oil Cooler</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
       </c>
-      <c r="E22" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -994,20 +1072,23 @@
           <t>Turbine Hall</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
         <is>
           <t>Turbine Lube Oil Pump</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
         <is>
           <t>Flow</t>
         </is>
       </c>
-      <c r="E23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1018,20 +1099,23 @@
           <t>Compressor House</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
         <is>
           <t>Compressor Discharge Pressure Indicator</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1042,20 +1126,23 @@
           <t>Compressor House</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
         <is>
           <t>Compressor Suction Temperature Gauge</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
       </c>
-      <c r="E25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1066,20 +1153,23 @@
           <t>Compressor House</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
         <is>
           <t>Instrument Air Receiver</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E26" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1090,20 +1180,23 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
         <is>
           <t>Chiller Unit 2</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
       </c>
-      <c r="E27" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" t="inlineStr">
         <is>
           <t>Chiller is not mapped</t>
         </is>
@@ -1118,20 +1211,23 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
         <is>
           <t>Fire Water Pump</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1143,15 +1239,18 @@
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr">
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="E29" t="n">
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="n">
         <v>0</v>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>empty description - nothing to convert</t>
         </is>
@@ -1166,20 +1265,23 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
         <is>
           <t>Emergency Diesel Generator</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="E30" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" t="inlineStr">
         <is>
           <t>Diesel/Generator are not mapped</t>
         </is>

</xml_diff>